<commit_message>
feat(dossier-cfa): isole les achats faits pour le compte de la société
Dans les notes de frais d'Anthony GRANDCLEMENT, séparation des deux natures :
4 097,01 € d'achats réglés chez un tiers puis remboursés (Bolt, Supabase,
Digiforma, Anthropic) contre 13 052,03 € d'indemnités kilométriques, péages,
repas et logement.

Chaque achat est nommé quand la source le permet, et l'onglet montre que ces
mêmes fournisseurs sont par ailleurs facturés en direct à la société — deux
canaux de règlement pour un même prestataire.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USnaW2gM3X4DgNMWJyXPCH
</commit_message>
<xml_diff>
--- a/dossier-cfa/livrables/Notes_de_frais_WEFORM.xlsx
+++ b/dossier-cfa/livrables/Notes_de_frais_WEFORM.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Règlements" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Lignes de charge" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Achats pour compte" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Notes'!$A$3:$G$63</definedName>
@@ -28,7 +29,7 @@
     <numFmt numFmtId="165" formatCode="# ##0.00;[Red]-# ##0.00;&quot;·&quot;"/>
     <numFmt numFmtId="166" formatCode="0.00&quot; %&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,6 +76,11 @@
       <i val="1"/>
       <color rgb="0078837F"/>
       <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00A8412C"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="4">
@@ -131,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,6 +187,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -549,7 +567,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
@@ -869,7 +887,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G63"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -2873,7 +2891,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E64"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -4424,7 +4442,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F88"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -6988,4 +7006,372 @@
   <autoFilter ref="A3:F88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="86" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Les notes de frais qui remboursent un achat fait chez un tiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>À distinguer des indemnités kilométriques : ici le salarié a payé un fournisseur de sa poche, et la facture est à son nom, pas à celui de la société.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Libellé du grand livre</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Montant</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Entité derrière la dépense</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Comment on le sait</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>30/04/2025</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS GRANDCLEMENT A 04.2026 APPLICATION</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>439.63</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Bolt + Supabase</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>« Douze lignes BOLT + SUPABASE sur la note d'avril 2025, aucun kilomètre » (dossier de synthèse WE-FORM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>31/05/2025</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS GRANDCLEMENT BOLT + ABO + DIGIFORMA</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>311.2</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Bolt 88,00 + Digiforma 223,20</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>« BOLT - ABO MAI - 100$ » 88,00 € et « DIGIFORMA » 223,20 € (dossier de synthèse WE-FORM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>04/08/2025</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS ANTHONY G 08.2025 SUPABASE (AVANCE)</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>1508.17</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Le libellé du grand livre le nomme : « SUPABASE (AVANCE) ». Votre modèle : « VIR INST SUPABASE — Base de données We-Admin ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>30/04/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS ANTHONY G 04.2026 ABONNEMT LOGICI IA</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>738.01</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Anthropic — API Claude</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Votre modèle isole « Note de frais avril — part API Claude » pour 738,00 €.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS ANTHONY G 07.2026 AVANCE FRAIS IA</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>Non identifiée</t>
+        </is>
+      </c>
+      <c r="E9" s="22" t="inlineStr">
+        <is>
+          <t>Libellé « AVANCE FRAIS IA ». Aucune entité nommée, ni au grand livre ni au modèle analytique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr"/>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Total des achats faits pour le compte de la société</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>4097.01</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr"/>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Ses notes de frais, en deux blocs</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Montant</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Achats payés chez un tiers et remboursés (logiciels, abonnements)</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>4097.01</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>23.89</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Indemnités kilométriques, péages, repas et logement</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>13052.03</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>76.11</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Total des notes de frais d'Anthony GRANDCLEMENT</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>17149.04</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Ces fournisseurs sont aussi facturés en direct</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Facturé en direct</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Via note de frais</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Remarque</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Bolt (StackBlitz)</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>2016.92</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>88</v>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Plus une part indéterminée des 439,63 € de la note d'avril 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>87.97</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>1508.17</v>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>1 508,17 € remboursés à Anthony contre 87,97 € facturés en direct : l'essentiel de la dépense passe par lui.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>1296.36</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>738.01</v>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Plus, peut-être, les 1 100 € de « AVANCE FRAIS IA » de juillet 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Digiforma</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>1951.2</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>223.2</v>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>Le direct passe par A World For Us (prélèvement GoCardless).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Un même fournisseur réglé par deux canaux : c'est le point à traiter. Quand la facture est au nom d'Anthony GRANDCLEMENT, la société perd la TVA déductible et la charge ne tient que par la note de frais. Le plus simple est de basculer ces abonnements sur un moyen de paiement de la société, comme cela a déjà été fait pour la part facturée en direct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>À part : la note du 06/12/2025, « TRANSPORT "RT" (A JUSTIFIER) » pour 314,00 €. La mention « à justifier » est du cabinet lui-même, elle figure telle quelle au grand livre.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A24:D24"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>